<commit_message>
Update Sprint 3 backlog
</commit_message>
<xml_diff>
--- a/documentation/scrum/Sprint_3_Backlog.xlsx
+++ b/documentation/scrum/Sprint_3_Backlog.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\imashai\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://micloud365-my.sharepoint.com/personal/imashai_millenniumitesp_com/Documents/Desktop/MSc BInA/Academics/3-Interactive Visualization/Assesment/Project/group4-interactive-visualisation/documentation/scrum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E3582D-88BE-45C0-B2FD-208A42EB60BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{E3E3582D-88BE-45C0-B2FD-208A42EB60BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D32C5D1B-EAFD-474B-BFE9-EA52676A4497}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="100">
   <si>
     <t>CIS4014-N Interactive Visualisation – Group 4 | Sprint 3 – Week 03</t>
   </si>
@@ -322,6 +322,9 @@
   </si>
   <si>
     <t>https://github.com/inkymello/group4-interactive-visualisation/blob/main/documentation/design/UI_Design_Document.docx</t>
+  </si>
+  <si>
+    <t>https://github.com/inkymello/group4-interactive-visualisation/blob/main/documentation/design/Interactive_Features_Added_Value.xlsx</t>
   </si>
 </sst>
 </file>
@@ -398,7 +401,6 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -420,6 +422,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -665,515 +668,521 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="6" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="D12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="I12" s="5"/>
+      <c r="I12" s="4"/>
     </row>
     <row r="13" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F13" s="4" t="s">
+      <c r="D13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="I13" s="5"/>
+      <c r="I13" s="4"/>
     </row>
     <row r="14" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F14" s="4" t="s">
+      <c r="D14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="5"/>
+      <c r="I14" s="4"/>
     </row>
     <row r="15" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F15" s="4" t="s">
+      <c r="D15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H15" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="I15" s="5"/>
+      <c r="I15" s="9" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F16" s="4" t="s">
+      <c r="D16" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="I16" s="5" t="s">
+      <c r="I16" s="4" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F17" s="4" t="s">
+      <c r="D17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="H17" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="I17" s="5"/>
+      <c r="I17" s="4"/>
     </row>
     <row r="18" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F18" s="4" t="s">
+      <c r="D18" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="I18" s="5"/>
+      <c r="I18" s="9" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F19" s="4" t="s">
+      <c r="D19" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="I19" s="5"/>
+      <c r="I19" s="4"/>
     </row>
     <row r="20" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F20" s="4" t="s">
+      <c r="D20" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H20" s="4" t="s">
+      <c r="H20" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="I20" s="5"/>
+      <c r="I20" s="4"/>
     </row>
     <row r="21" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F21" s="4" t="s">
+      <c r="D21" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H21" s="4" t="s">
+      <c r="H21" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I21" s="5"/>
+      <c r="I21" s="9" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="22" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F22" s="4" t="s">
+      <c r="D22" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="I22" s="9" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F23" s="4" t="s">
+      <c r="D23" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="I23" s="5"/>
+      <c r="I23" s="4"/>
     </row>
     <row r="24" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F24" s="4" t="s">
+      <c r="D24" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="I24" s="5"/>
+      <c r="I24" s="4"/>
     </row>
     <row r="25" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F25" s="4" t="s">
+      <c r="D25" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="H25" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="I25" s="5"/>
+      <c r="I25" s="4"/>
     </row>
     <row r="26" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F26" s="4" t="s">
+      <c r="D26" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H26" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="I26" s="5" t="s">
+      <c r="I26" s="4" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="I27" s="9"/>
+      <c r="I27" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1181,11 +1190,14 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I22" r:id="rId1" xr:uid="{6CBB444F-E011-458A-8585-D6C3A3F3BB47}"/>
+    <hyperlink ref="I15" r:id="rId2" xr:uid="{C94440C1-0A3B-4447-B4AD-2DCA82E5360A}"/>
+    <hyperlink ref="I18" r:id="rId3" xr:uid="{A37AFD02-6958-4DAD-94B0-9516928B6ABD}"/>
+    <hyperlink ref="I21" r:id="rId4" xr:uid="{BF40E71E-A945-43BE-9F5C-327FFF10FDA2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Sprint 4 scrum documentation
</commit_message>
<xml_diff>
--- a/documentation/scrum/Sprint_3_Backlog.xlsx
+++ b/documentation/scrum/Sprint_3_Backlog.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://micloud365-my.sharepoint.com/personal/imashai_millenniumitesp_com/Documents/Desktop/MSc BInA/Academics/3-Interactive Visualization/Assesment/Project/group4-interactive-visualisation/documentation/scrum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{E3E3582D-88BE-45C0-B2FD-208A42EB60BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D32C5D1B-EAFD-474B-BFE9-EA52676A4497}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{E3E3582D-88BE-45C0-B2FD-208A42EB60BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D05D3E9-A64D-4435-854D-32BD1470F706}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint 3" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="103">
   <si>
     <t>CIS4014-N Interactive Visualisation – Group 4 | Sprint 3 – Week 03</t>
   </si>
@@ -165,9 +165,6 @@
     <t>D3.js Store Location Map with ranked store detail</t>
   </si>
   <si>
-    <t>Chart 2 ownership unchanged since Sprint 2 — Ilamperuma.</t>
-  </si>
-  <si>
     <t>S3-06</t>
   </si>
   <si>
@@ -325,6 +322,18 @@
   </si>
   <si>
     <t>https://github.com/inkymello/group4-interactive-visualisation/blob/main/documentation/design/Interactive_Features_Added_Value.xlsx</t>
+  </si>
+  <si>
+    <t>https://github.com/inkymello/group4-interactive-visualisation/tree/main/dashboard/initial%20dashbaord</t>
+  </si>
+  <si>
+    <t>https://github.com/inkymello/group4-interactive-visualisation/tree/main/charts/De%20Silva</t>
+  </si>
+  <si>
+    <t>https://github.com/inkymello/group4-interactive-visualisation/tree/main/charts/Ilamperuma</t>
+  </si>
+  <si>
+    <t>https://github.com/inkymello/group4-interactive-visualisation/tree/main/charts/Samarakoon</t>
   </si>
 </sst>
 </file>
@@ -399,7 +408,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -423,6 +432,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -454,6 +466,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -784,10 +800,10 @@
         <v>29</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I12" s="4"/>
     </row>
@@ -814,9 +830,11 @@
         <v>34</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="I13" s="4"/>
+        <v>83</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -841,7 +859,7 @@
         <v>38</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I14" s="4"/>
     </row>
@@ -868,10 +886,10 @@
         <v>38</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -897,18 +915,18 @@
         <v>34</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>46</v>
+        <v>86</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>48</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>44</v>
@@ -920,22 +938,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>38</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I17" s="4"/>
     </row>
     <row r="18" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>51</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>44</v>
@@ -947,107 +965,109 @@
         <v>28</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>38</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>57</v>
-      </c>
       <c r="H19" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="I19" s="4"/>
+        <v>89</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="20" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="C20" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>59</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>60</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>38</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I20" s="4"/>
     </row>
     <row r="21" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="C21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>63</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>38</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>65</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>26</v>
@@ -1059,24 +1079,24 @@
         <v>28</v>
       </c>
       <c r="F22" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G22" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G22" s="3" t="s">
-        <v>67</v>
-      </c>
       <c r="H22" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>69</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>26</v>
@@ -1088,22 +1108,24 @@
         <v>28</v>
       </c>
       <c r="F23" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G23" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G23" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="H23" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I23" s="4"/>
+        <v>93</v>
+      </c>
+      <c r="I23" s="11" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="24" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>26</v>
@@ -1115,22 +1137,22 @@
         <v>28</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I24" s="4"/>
     </row>
     <row r="25" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>76</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>26</v>
@@ -1142,22 +1164,22 @@
         <v>28</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I25" s="4"/>
     </row>
     <row r="26" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>26</v>
@@ -1169,16 +1191,16 @@
         <v>28</v>
       </c>
       <c r="F26" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G26" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="H26" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="I26" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
@@ -1193,11 +1215,15 @@
     <hyperlink ref="I15" r:id="rId2" xr:uid="{C94440C1-0A3B-4447-B4AD-2DCA82E5360A}"/>
     <hyperlink ref="I18" r:id="rId3" xr:uid="{A37AFD02-6958-4DAD-94B0-9516928B6ABD}"/>
     <hyperlink ref="I21" r:id="rId4" xr:uid="{BF40E71E-A945-43BE-9F5C-327FFF10FDA2}"/>
+    <hyperlink ref="I23" r:id="rId5" xr:uid="{D2D2838E-FC66-437C-808F-B353C15AFF49}"/>
+    <hyperlink ref="I19" r:id="rId6" xr:uid="{F100A16D-DB84-4839-B3EA-2FDCD1E37F7A}"/>
+    <hyperlink ref="I16" r:id="rId7" xr:uid="{A753DAD4-8004-4BF3-9EC6-FE7B36A98C9E}"/>
+    <hyperlink ref="I13" r:id="rId8" xr:uid="{3BA83849-9A24-4476-9E69-E25634D55FBE}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Sprint 3 and Sprint 4 documentation
</commit_message>
<xml_diff>
--- a/documentation/scrum/Sprint_3_Backlog.xlsx
+++ b/documentation/scrum/Sprint_3_Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://micloud365-my.sharepoint.com/personal/imashai_millenniumitesp_com/Documents/Desktop/MSc BInA/Academics/3-Interactive Visualization/Assesment/Project/group4-interactive-visualisation/documentation/scrum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{E3E3582D-88BE-45C0-B2FD-208A42EB60BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D05D3E9-A64D-4435-854D-32BD1470F706}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{E3E3582D-88BE-45C0-B2FD-208A42EB60BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75E5725A-CD2C-47BF-9836-97F16FD58A75}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -324,9 +324,6 @@
     <t>https://github.com/inkymello/group4-interactive-visualisation/blob/main/documentation/design/Interactive_Features_Added_Value.xlsx</t>
   </si>
   <si>
-    <t>https://github.com/inkymello/group4-interactive-visualisation/tree/main/dashboard/initial%20dashbaord</t>
-  </si>
-  <si>
     <t>https://github.com/inkymello/group4-interactive-visualisation/tree/main/charts/De%20Silva</t>
   </si>
   <si>
@@ -334,6 +331,9 @@
   </si>
   <si>
     <t>https://github.com/inkymello/group4-interactive-visualisation/tree/main/charts/Samarakoon</t>
+  </si>
+  <si>
+    <t>https://github.com/inkymello/group4-interactive-visualisation/tree/main/dashboard/initial%20dashboard</t>
   </si>
 </sst>
 </file>
@@ -431,10 +431,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -684,16 +684,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -832,8 +832,8 @@
       <c r="H13" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="I13" s="11" t="s">
-        <v>102</v>
+      <c r="I13" s="10" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -917,8 +917,8 @@
       <c r="H16" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="11" t="s">
-        <v>101</v>
+      <c r="I16" s="10" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1002,8 +1002,8 @@
       <c r="H19" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="I19" s="11" t="s">
-        <v>100</v>
+      <c r="I19" s="10" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1116,8 +1116,8 @@
       <c r="H23" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="I23" s="11" t="s">
-        <v>99</v>
+      <c r="I23" s="10" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>